<commit_message>
feat: initialize competition data, implement database seeder, and update competition schema and pages
</commit_message>
<xml_diff>
--- a/src/assets/dokumen/Arena Inovasi Digital/TIMELINE LOMBA.xlsx
+++ b/src/assets/dokumen/Arena Inovasi Digital/TIMELINE LOMBA.xlsx
@@ -79,13 +79,13 @@
     <t>Pendaftaran : Gelombang I</t>
   </si>
   <si>
-    <t xml:space="preserve">5 Juli - 15 Juli </t>
+    <t xml:space="preserve">9 Juli - 17 Juli </t>
   </si>
   <si>
     <t xml:space="preserve">Pendaftaran : Gelombang II </t>
   </si>
   <si>
-    <t>16 Juli - 5 Agustus</t>
+    <t>18 Juli - 9 Agustus</t>
   </si>
   <si>
     <t>Technical Meeting</t>
@@ -97,7 +97,7 @@
     <t>Penilaian Awal</t>
   </si>
   <si>
-    <t>25 - 31 Agustus</t>
+    <t>29 - 3September</t>
   </si>
   <si>
     <t>Pengumuman Top 5</t>
@@ -124,7 +124,7 @@
     <t>Mentoring</t>
   </si>
   <si>
-    <t>Infokan Hanna Asa</t>
+    <t>Infokan Hannah Asa</t>
   </si>
   <si>
     <t>Final</t>
@@ -340,7 +340,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="40">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -428,6 +428,9 @@
     <xf borderId="2" fillId="0" fontId="5" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="14" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="14" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="14" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment readingOrder="0"/>
@@ -976,7 +979,7 @@
       <c r="B23" s="23" t="s">
         <v>19</v>
       </c>
-      <c r="C23" s="22" t="s">
+      <c r="C23" s="15" t="s">
         <v>20</v>
       </c>
     </row>
@@ -1003,7 +1006,7 @@
         <v>25</v>
       </c>
       <c r="B26" s="26">
-        <v>46240.0</v>
+        <v>46244.0</v>
       </c>
       <c r="C26" s="18"/>
     </row>
@@ -1012,7 +1015,7 @@
         <v>26</v>
       </c>
       <c r="B27" s="26">
-        <v>46258.0</v>
+        <v>46262.0</v>
       </c>
       <c r="C27" s="18"/>
       <c r="F27" s="27"/>
@@ -1031,7 +1034,7 @@
         <v>29</v>
       </c>
       <c r="B29" s="28">
-        <v>46266.0</v>
+        <v>46269.0</v>
       </c>
       <c r="C29" s="18"/>
     </row>
@@ -1040,7 +1043,7 @@
         <v>30</v>
       </c>
       <c r="B30" s="26">
-        <v>46268.0</v>
+        <v>46273.0</v>
       </c>
       <c r="C30" s="18"/>
     </row>
@@ -1049,7 +1052,7 @@
         <v>31</v>
       </c>
       <c r="B31" s="28">
-        <v>46272.0</v>
+        <v>46277.0</v>
       </c>
       <c r="C31" s="18"/>
     </row>
@@ -1074,7 +1077,7 @@
       <c r="B35" s="23" t="s">
         <v>19</v>
       </c>
-      <c r="C35" s="22" t="s">
+      <c r="C35" s="15" t="s">
         <v>20</v>
       </c>
     </row>
@@ -1101,7 +1104,7 @@
         <v>34</v>
       </c>
       <c r="B38" s="26">
-        <v>46241.0</v>
+        <v>46245.0</v>
       </c>
       <c r="C38" s="18"/>
     </row>
@@ -1110,7 +1113,7 @@
         <v>35</v>
       </c>
       <c r="B39" s="26">
-        <v>46258.0</v>
+        <v>46262.0</v>
       </c>
       <c r="C39" s="18"/>
     </row>
@@ -1119,7 +1122,7 @@
         <v>29</v>
       </c>
       <c r="B40" s="26">
-        <v>46266.0</v>
+        <v>46269.0</v>
       </c>
       <c r="C40" s="18"/>
     </row>
@@ -1137,7 +1140,7 @@
         <v>38</v>
       </c>
       <c r="B42" s="28">
-        <v>46272.0</v>
+        <v>46276.0</v>
       </c>
       <c r="C42" s="18"/>
     </row>
@@ -1167,7 +1170,7 @@
       <c r="B46" s="23" t="s">
         <v>19</v>
       </c>
-      <c r="C46" s="22" t="s">
+      <c r="C46" s="38" t="s">
         <v>20</v>
       </c>
     </row>
@@ -1194,16 +1197,16 @@
         <v>25</v>
       </c>
       <c r="B49" s="26">
-        <v>46242.0</v>
+        <v>46246.0</v>
       </c>
       <c r="C49" s="18"/>
     </row>
     <row r="50">
-      <c r="A50" s="38" t="s">
+      <c r="A50" s="39" t="s">
         <v>39</v>
       </c>
       <c r="B50" s="26">
-        <v>46258.0</v>
+        <v>46262.0</v>
       </c>
       <c r="C50" s="18"/>
     </row>
@@ -1212,7 +1215,7 @@
         <v>29</v>
       </c>
       <c r="B51" s="28">
-        <v>46266.0</v>
+        <v>46269.0</v>
       </c>
       <c r="C51" s="18"/>
     </row>
@@ -1237,7 +1240,7 @@
       <c r="B55" s="23" t="s">
         <v>19</v>
       </c>
-      <c r="C55" s="22" t="s">
+      <c r="C55" s="15" t="s">
         <v>20</v>
       </c>
     </row>
@@ -1264,7 +1267,7 @@
         <v>25</v>
       </c>
       <c r="B58" s="26">
-        <v>46244.0</v>
+        <v>46248.0</v>
       </c>
       <c r="C58" s="18"/>
     </row>
@@ -1273,7 +1276,7 @@
         <v>40</v>
       </c>
       <c r="B59" s="26">
-        <v>46258.0</v>
+        <v>46262.0</v>
       </c>
       <c r="C59" s="18"/>
     </row>
@@ -1282,7 +1285,7 @@
         <v>29</v>
       </c>
       <c r="B60" s="28">
-        <v>46235.0</v>
+        <v>46269.0</v>
       </c>
       <c r="C60" s="18"/>
     </row>
@@ -1307,7 +1310,7 @@
       <c r="B64" s="23" t="s">
         <v>19</v>
       </c>
-      <c r="C64" s="22" t="s">
+      <c r="C64" s="15" t="s">
         <v>20</v>
       </c>
     </row>
@@ -1334,7 +1337,7 @@
         <v>25</v>
       </c>
       <c r="B67" s="26">
-        <v>46245.0</v>
+        <v>46249.0</v>
       </c>
       <c r="C67" s="18"/>
     </row>
@@ -1343,7 +1346,7 @@
         <v>42</v>
       </c>
       <c r="B68" s="26">
-        <v>46247.0</v>
+        <v>46251.0</v>
       </c>
       <c r="C68" s="18"/>
     </row>
@@ -1352,7 +1355,7 @@
         <v>43</v>
       </c>
       <c r="B69" s="26">
-        <v>46258.0</v>
+        <v>46262.0</v>
       </c>
       <c r="C69" s="18"/>
     </row>
@@ -1361,7 +1364,7 @@
         <v>29</v>
       </c>
       <c r="B70" s="28">
-        <v>46266.0</v>
+        <v>46269.0</v>
       </c>
       <c r="C70" s="18"/>
     </row>
@@ -1370,7 +1373,7 @@
         <v>38</v>
       </c>
       <c r="B71" s="28">
-        <v>46268.0</v>
+        <v>46270.0</v>
       </c>
       <c r="C71" s="18"/>
     </row>

</xml_diff>